<commit_message>
DOI - Klaar ?
</commit_message>
<xml_diff>
--- a/Antithetic_Results_Rule1.xlsx
+++ b/Antithetic_Results_Rule1.xlsx
@@ -444,13 +444,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>22.57261387754749</v>
+        <v>74.37361187111355</v>
       </c>
       <c r="C2" t="n">
-        <v>2.907346466947512</v>
+        <v>2.084880238497711</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4573992932176649</v>
+        <v>0.6743534304944692</v>
       </c>
     </row>
   </sheetData>
@@ -494,13 +494,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>24.83298621384904</v>
+        <v>26.75422267957043</v>
       </c>
       <c r="C2" t="n">
-        <v>2.912451916194826</v>
+        <v>2.087110509044544</v>
       </c>
       <c r="D2" t="n">
-        <v>0.4714211625961455</v>
+        <v>0.3911524931452495</v>
       </c>
     </row>
   </sheetData>

</xml_diff>